<commit_message>
feat: add basic tutorial
</commit_message>
<xml_diff>
--- a/tutorial/Horario_Tesis.xlsx
+++ b/tutorial/Horario_Tesis.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -450,7 +450,6 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,7 +466,6 @@
       <c r="K1" t="inlineStr"/>
       <c r="L1" t="inlineStr"/>
       <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -483,47 +481,46 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Estudiante</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Tutor</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Presidente</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Secretario</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Vocal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Oponente</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Presidente</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Vocal</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Secretario</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Dia</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Hora</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -539,306 +536,1203 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Grado</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
           <t>Defensas</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Juan Diaz</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Piad</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Angel Daniel Alonso Guevara</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Lopez</t>
+          <t>MSc. Carmen T. Fernández Montoto</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Torres</t>
+          <t>Dr. Alberto Fernández Oliva</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>Ruiz</t>
+          <t>Lic. Alejandro Labourdette-Lantigua Soto</t>
         </is>
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Lunes</t>
+          <t>Lic. Dennis Daniel González Durán</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>MSc. Aracelys García Armenteros</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>Aula 1</t>
+          <t>Postgrado</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>Piad</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="inlineStr">
-        <is>
-          <t>Dr</t>
-        </is>
-      </c>
-      <c r="M4" s="1">
-        <f>COUNTIF($B$4:$F$6,K4)</f>
-        <v/>
-      </c>
-      <c r="N4" t="inlineStr"/>
+          <t>Dr. Alberto Fernández Oliva</t>
+        </is>
+      </c>
+      <c r="L4" s="1">
+        <f>COUNTIF($D$4:$H$16,K4)</f>
+        <v/>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Maria Vega</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Lopez</t>
+          <t>Adrián Hernández Castellanos</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Piad</t>
+          <t>Lic. Alejandra Monzón Peña</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Soto</t>
+          <t>Lic. Amanda Noris Hernández</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>Torres</t>
+          <t>Lic. Kevin Manzano Rodríguez</t>
         </is>
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>Lunes</t>
+          <t>Lic. Daniel Abad Fundora</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>Lic. Rodrigo García Gómez</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>Aula 2</t>
+          <t>Salón decanato</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" s="1" t="inlineStr">
         <is>
-          <t>Garcia</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="inlineStr">
-        <is>
-          <t>Dr</t>
-        </is>
-      </c>
-      <c r="M5" s="1">
-        <f>COUNTIF($B$4:$F$6,K5)</f>
-        <v/>
-      </c>
-      <c r="N5" t="inlineStr"/>
+          <t>Dr. Gabriel Fundora</t>
+        </is>
+      </c>
+      <c r="L5" s="1">
+        <f>COUNTIF($D$4:$H$16,K5)</f>
+        <v/>
+      </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Luis Mora</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Lopez</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Torres</t>
+          <t>Laura Martir Beltrán</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Lic. Alejandra Monzón Peña</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Ruiz</t>
+          <t>Lic. Amanda Noris Hernández</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>Soto</t>
+          <t>Lic. Kevin Manzano Rodríguez</t>
         </is>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>Lunes</t>
+          <t>Lic. Daniel Abad Fundora</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>Lic. Rodrigo García Gómez</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
         <is>
-          <t>Aula 3</t>
+          <t>Salón decanato</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" s="1" t="inlineStr">
         <is>
-          <t>Lopez</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="M6" s="1">
-        <f>COUNTIF($B$4:$F$6,K6)</f>
-        <v/>
-      </c>
-      <c r="N6" t="inlineStr"/>
+          <t>DrC. Alejandro Piad Morfis</t>
+        </is>
+      </c>
+      <c r="L6" s="1">
+        <f>COUNTIF($D$4:$H$16,K6)</f>
+        <v/>
+      </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7">
-        <f>"Total defensas:"</f>
-        <v/>
-      </c>
-      <c r="B7">
-        <f>COUNTA($A$4:$A$6)</f>
-        <v/>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Noel Pérez Calvo</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Fernando Raúl Rodríguez Flores</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Rodrigo García Gómez</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Lázaro Daniel González Martínez</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandra Monzón Peña</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>Lic. David Guaty Domínguez</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>Salón decanato</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>Torres</t>
-        </is>
-      </c>
-      <c r="L7" s="1" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="M7" s="1">
-        <f>COUNTIF($B$4:$F$6,K7)</f>
-        <v/>
-      </c>
-      <c r="N7" t="inlineStr"/>
+          <t>DrC. Alejandro Sánchez Castellanos</t>
+        </is>
+      </c>
+      <c r="L7" s="1">
+        <f>COUNTIF($D$4:$H$16,K7)</f>
+        <v/>
+      </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Claudia Hernández Pérez y Joel Aparicio Tamayo</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Celia T. González González</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Dra. Ayme Marrero Severo</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Joanna Campbell Amos</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Daniel Alejandro Valdés Pérez</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Beltrán Varela</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Postgrado</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>Ruiz</t>
-        </is>
-      </c>
-      <c r="L8" s="1" t="inlineStr">
-        <is>
-          <t>Lic</t>
-        </is>
-      </c>
-      <c r="M8" s="1">
-        <f>COUNTIF($B$4:$F$6,K8)</f>
-        <v/>
-      </c>
-      <c r="N8" t="inlineStr"/>
+          <t>Dra. Ayme Marrero Severo</t>
+        </is>
+      </c>
+      <c r="L8" s="1">
+        <f>COUNTIF($D$4:$H$16,K8)</f>
+        <v/>
+      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Darío Hernández Cubilla</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Aracelys García Armenteros</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Dra. Ayme Marrero Severo</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Roberto Marti Cedeño</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Beltrán Varela</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Labourdette-Lantigua Soto</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>Postgrado</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>Soto</t>
-        </is>
-      </c>
-      <c r="L9" s="1" t="inlineStr">
-        <is>
-          <t>Msc</t>
-        </is>
-      </c>
-      <c r="M9" s="1">
-        <f>COUNTIF($B$4:$F$6,K9)</f>
-        <v/>
-      </c>
-      <c r="N9" t="inlineStr"/>
+          <t>DraC. Marta Lourdes Baguer Díaz-Romañach</t>
+        </is>
+      </c>
+      <c r="L9" s="1">
+        <f>COUNTIF($D$4:$H$16,K9)</f>
+        <v/>
+      </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="K10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Richard Alejandro Matos Arderí</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Celia T. González González</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Wilfredo Morales Lezca</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Roberto Marti Cedeño</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Beltrán Varela</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Aracelys García Armenteros</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>Postgrado</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandra Monzón Peña</t>
+        </is>
+      </c>
+      <c r="L10" s="1">
+        <f>COUNTIF($D$4:$H$16,K10)</f>
+        <v/>
+      </c>
+      <c r="M10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Melani Forsythe Matos</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>DraC. Marta Lourdes Baguer Díaz-Romañach</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>DrC. Alejandro Sánchez Castellanos</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Ana Paula González Muñoz</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Dennis Daniel González Durán</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Javier Rodríguez Sánchez</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>Francofonía</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Beltrán Varela</t>
+        </is>
+      </c>
+      <c r="L11" s="1">
+        <f>COUNTIF($D$4:$H$16,K11)</f>
+        <v/>
+      </c>
+      <c r="M11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Mauro Eduardo Campver Barrios</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>DraC. Marta Lourdes Baguer Díaz-Romañach</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>DrC. Alejandro Piad Morfis</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Ana Paula González Muñoz</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Dennis Daniel González Durán</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Fernando Raúl Rodríguez Flores</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Francofonía</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Labourdette-Lantigua Soto</t>
+        </is>
+      </c>
+      <c r="L12" s="1">
+        <f>COUNTIF($D$4:$H$16,K12)</f>
+        <v/>
+      </c>
+      <c r="M12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>José Miguel Leyva De La Cruz</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Beltrán Varela</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Amanda Noris Hernández</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Juan Miguel Pérez Martínez</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Fundora</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Aracelys García Armenteros</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>Francofonía</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Amanda Noris Hernández</t>
+        </is>
+      </c>
+      <c r="L13" s="1">
+        <f>COUNTIF($D$4:$H$16,K13)</f>
+        <v/>
+      </c>
+      <c r="M13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Jossué Arteche Muñoz</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Fernando Raúl Rodríguez Flores</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>DrC. Alejandro Piad Morfis</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Rodrigo García Gómez</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Daniel Abad Fundora</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Ariel González Gómez</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Salón decanato</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Ana Paula González Muñoz</t>
+        </is>
+      </c>
+      <c r="L14" s="1">
+        <f>COUNTIF($D$4:$H$16,K14)</f>
+        <v/>
+      </c>
+      <c r="M14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Amalia Beatriz Valiente Hinojosa</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Fernando Raúl Rodríguez Flores</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Javier Rodríguez Sánchez</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Rocío Ortiz Gancedo</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Merling Sabater Ramírez</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandra Monzón Peña</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>Salón decanato</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Ariel González Gómez</t>
+        </is>
+      </c>
+      <c r="L15" s="1">
+        <f>COUNTIF($D$4:$H$16,K15)</f>
+        <v/>
+      </c>
+      <c r="M15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Luis Ernesto Amat Cárdenas</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Roberto Marti Cedeño</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>DrC. Alejandro Piad Morfis</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Carlos David Muñiz Chall</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Alejandro Labourdette-Lantigua Soto</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Daniel Toledo Martínez</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Salón decanato</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Carlos David Muñiz Chall</t>
+        </is>
+      </c>
+      <c r="L16" s="1">
+        <f>COUNTIF($D$4:$H$16,K16)</f>
+        <v/>
+      </c>
+      <c r="M16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>"Total defensas:"</f>
+        <v/>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17">
+        <f>COUNTA($C$4:$C$16)</f>
+        <v/>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Daniel Abad Fundora</t>
+        </is>
+      </c>
+      <c r="L17" s="1">
+        <f>COUNTIF($D$4:$H$16,K17)</f>
+        <v/>
+      </c>
+      <c r="M17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Daniel Alejandro Valdés Pérez</t>
+        </is>
+      </c>
+      <c r="L18" s="1">
+        <f>COUNTIF($D$4:$H$16,K18)</f>
+        <v/>
+      </c>
+      <c r="M18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Daniel Toledo Martínez</t>
+        </is>
+      </c>
+      <c r="L19" s="1">
+        <f>COUNTIF($D$4:$H$16,K19)</f>
+        <v/>
+      </c>
+      <c r="M19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>Lic. David Guaty Domínguez</t>
+        </is>
+      </c>
+      <c r="L20" s="1">
+        <f>COUNTIF($D$4:$H$16,K20)</f>
+        <v/>
+      </c>
+      <c r="M20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Dennis Daniel González Durán</t>
+        </is>
+      </c>
+      <c r="L21" s="1">
+        <f>COUNTIF($D$4:$H$16,K21)</f>
+        <v/>
+      </c>
+      <c r="M21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Javier Rodríguez Sánchez</t>
+        </is>
+      </c>
+      <c r="L22" s="1">
+        <f>COUNTIF($D$4:$H$16,K22)</f>
+        <v/>
+      </c>
+      <c r="M22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Juan Miguel Pérez Martínez</t>
+        </is>
+      </c>
+      <c r="L23" s="1">
+        <f>COUNTIF($D$4:$H$16,K23)</f>
+        <v/>
+      </c>
+      <c r="M23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Kevin Manzano Rodríguez</t>
+        </is>
+      </c>
+      <c r="L24" s="1">
+        <f>COUNTIF($D$4:$H$16,K24)</f>
+        <v/>
+      </c>
+      <c r="M24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Lázaro Daniel González Martínez</t>
+        </is>
+      </c>
+      <c r="L25" s="1">
+        <f>COUNTIF($D$4:$H$16,K25)</f>
+        <v/>
+      </c>
+      <c r="M25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Merling Sabater Ramírez</t>
+        </is>
+      </c>
+      <c r="L26" s="1">
+        <f>COUNTIF($D$4:$H$16,K26)</f>
+        <v/>
+      </c>
+      <c r="M26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Roberto Marti Cedeño</t>
+        </is>
+      </c>
+      <c r="L27" s="1">
+        <f>COUNTIF($D$4:$H$16,K27)</f>
+        <v/>
+      </c>
+      <c r="M27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Rocío Ortiz Gancedo</t>
+        </is>
+      </c>
+      <c r="L28" s="1">
+        <f>COUNTIF($D$4:$H$16,K28)</f>
+        <v/>
+      </c>
+      <c r="M28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" s="1" t="inlineStr">
+        <is>
+          <t>Lic. Rodrigo García Gómez</t>
+        </is>
+      </c>
+      <c r="L29" s="1">
+        <f>COUNTIF($D$4:$H$16,K29)</f>
+        <v/>
+      </c>
+      <c r="M29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Aracelys García Armenteros</t>
+        </is>
+      </c>
+      <c r="L30" s="1">
+        <f>COUNTIF($D$4:$H$16,K30)</f>
+        <v/>
+      </c>
+      <c r="M30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Carmen T. Fernández Montoto</t>
+        </is>
+      </c>
+      <c r="L31" s="1">
+        <f>COUNTIF($D$4:$H$16,K31)</f>
+        <v/>
+      </c>
+      <c r="M31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Celia T. González González</t>
+        </is>
+      </c>
+      <c r="L32" s="1">
+        <f>COUNTIF($D$4:$H$16,K32)</f>
+        <v/>
+      </c>
+      <c r="M32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Fernando Raúl Rodríguez Flores</t>
+        </is>
+      </c>
+      <c r="L33" s="1">
+        <f>COUNTIF($D$4:$H$16,K33)</f>
+        <v/>
+      </c>
+      <c r="M33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Joanna Campbell Amos</t>
+        </is>
+      </c>
+      <c r="L34" s="1">
+        <f>COUNTIF($D$4:$H$16,K34)</f>
+        <v/>
+      </c>
+      <c r="M34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" s="1" t="inlineStr">
+        <is>
+          <t>MSc. Wilfredo Morales Lezca</t>
+        </is>
+      </c>
+      <c r="L35" s="1">
+        <f>COUNTIF($D$4:$H$16,K35)</f>
+        <v/>
+      </c>
+      <c r="M35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="K36">
         <f>"Total profesores:"</f>
         <v/>
       </c>
-      <c r="M10">
-        <f>SUM($M$4:$M$9)</f>
+      <c r="L36">
+        <f>SUM($L$4:$L$35)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K4:K9">
+  <conditionalFormatting sqref="K4:K35">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
-      <formula>SUMPRODUCT((($B$4:$B$6=$K4)+($C$4:$C$6=$K4)+($D$4:$D$6=$K4)+($E$4:$E$6=$K4)+($F$4:$F$6=$K4))*(COUNTIFS($G$4:$G$6,$G$4:$G$6,$H$4:$H$6,$H$4:$H$6)&gt;1))&gt;0</formula>
+      <formula>SUMPRODUCT((($D$4:$D$16=$K4)+($E$4:$E$16=$K4)+($F$4:$F$16=$K4)+($G$4:$G$16=$K4)+($H$4:$H$16=$K4))*(COUNTIFS($A$4:$A$16,$A$4:$A$16,$B$4:$B$16,$B$4:$B$16)&gt;1))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>